<commit_message>
fix: remove duplicate line control tourism memo header in culture section
</commit_message>
<xml_diff>
--- a/scripts/Thai_Weekly_DB.xlsx
+++ b/scripts/Thai_Weekly_DB.xlsx
@@ -565,8 +565,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;💡 線控經理實務備忘（Line Control Tourism Memo）：&lt;/b&gt;&lt;br/&gt;
-        在觀光旅遊接待上，泰國對「素食」有極清晰的語義界線：&lt;br/&gt;
+          <t>在觀光旅遊接待上，泰國對「素食」有極清晰的語義界線：&lt;br/&gt;
         1. &lt;b&gt;กินเจ (Gin Jee - 齋戒純素)&lt;/b&gt;：必須完全無肉、無海鮮、無蛋奶、避五辛（蒜蔥洋蔥），且廚具嚴格分開。&lt;br/&gt;
         2. &lt;b&gt;มังสวิรัติ (Mang-sa-wí-rát - 蔬食/蛋奶素)&lt;/b&gt;：一般蔬食主義，多數可接受蔥蒜、蛋、乳製品，但不含肉塊。&lt;br/&gt;
         3. &lt;b&gt;團體餐食操作準則&lt;/b&gt;：遇台灣進香團、祈福團或茹素旅客赴泰，在向曼谷、芭達雅或清邁餐廳下訂單（Booking Request）時，務必精確註記是「อาหารเจ (Jay - 嚴格純素齋戒)」還是「มังสวิรัติ (Vegetarian - 蛋奶素)」，避免餐廳誤放蠔油、魚露或蔥蒜調味，確保高標準服務體驗！</t>
@@ -577,8 +576,6 @@
           <t>【泰語學習週報】VOL. 26w41 ｜ 飲食預訂實務・語法名詞化與九皇齋節文化誌</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -645,8 +642,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;💡 線控經理實務備忘（Line Control Tourism Memo）：&lt;/b&gt;&lt;br/&gt;
-        水燈節期間赴泰觀光熱潮達到年度最高峰，專業線控人員與隨團經理需嚴密落實以下營運細節：&lt;br/&gt;
+          <t>水燈節期間赴泰觀光熱潮達到年度最高峰，專業線控人員與隨團經理需嚴密落實以下營運細節：&lt;br/&gt;
         1. &lt;b&gt;交通動線防塞預案&lt;/b&gt;：水燈節當晚曼谷昭披耶河沿岸（如 ICONSIAM、Asiatique、鄭王廟、大皇宮）與清邁古城周遭運河將實施大範圍交管，陸路車流往往陷入數小時癱瘓。規劃團體或貴賓行程時，務必強制提前至少 2 小時動身，並優先包租專屬遊船或引導搭乘空鐵 BTS 至 Sathorn 碼頭轉乘專屬接駁船，徹底避開陸上壅塞。&lt;br/&gt;
         2. &lt;b&gt;景觀餐廳與遊船訂位&lt;/b&gt;：河畔五星飯店戶外座席與昭披耶河晚餐遊船（Dinner Cruise）通常於節慶前 1 至 2 個月即全數滿席。若有安排放水燈環節，需確認遊船甲板施放動線與救生防護規範，確保旅客在最安全雅緻的氛圍中深度領略泰式節慶之美！</t>
         </is>
@@ -656,8 +652,6 @@
           <t>【泰語學習週報】VOL. 26w42 ｜ 交通指引・機場退稅與水燈節前哨</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -724,8 +718,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;💡 線控經理實務備忘（Line Control Tourism Memo）：&lt;/b&gt;&lt;br/&gt;
-        在台泰觀光同業對接飯店房單（Rooming List）與現場領隊分房時，有一個極易踩雷的&lt;b&gt;「泰語房型字義陷阱」&lt;/b&gt;務必高度警惕：&lt;br/&gt;
+          <t>在台泰觀光同業對接飯店房單（Rooming List）與現場領隊分房時，有一個極易踩雷的&lt;b&gt;「泰語房型字義陷阱」&lt;/b&gt;務必高度警惕：&lt;br/&gt;
         1. &lt;b&gt;ห้องเตียงเดี่ยว (Hɔ̂ng dtiang dìaw)&lt;/b&gt;：字面直譯雖是「單床房」，但在泰國飯店術語中，指的卻是&lt;b&gt;「一張大床的雙人房（Double / King Size Bed Room）」&lt;/b&gt;（因為只有「一張」大床）！&lt;br/&gt;
         2. &lt;b&gt;ห้องเตียงคู่ (Hɔ̂ng dtiang khûu)&lt;/b&gt;：字面是「成對床房」，實務上才是台灣旅客習慣稱呼的&lt;b&gt;「兩張單人床房（Twin Room）」&lt;/b&gt;！&lt;br/&gt;
         3. &lt;b&gt;操作防呆準則&lt;/b&gt;：台灣團體旅客（如同事、朋友同住）極度要求「一人睡一張床（Twin Beds）」。向泰國 Local 地接社或飯店訂房組確認時，務必明確指定需要 &lt;b&gt;Twin Room (ห้องเตียงคู่ - 2 เตียง)&lt;/b&gt;，切勿因字面誤會訂成 &lt;code&gt;เตียงเดี่ยว&lt;/code&gt;，從源頭杜絕團體進房後的換房風波！</t>
@@ -801,12 +794,6 @@
           <t>9個核心單字 ｜ 5組日常對話 ｜ 2大核心語法 ｜ 泰式草藥醫學文化誌</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>